<commit_message>
Standardize channel colors across dashboard and exports
</commit_message>
<xml_diff>
--- a/public/downloads/Separate_July_Sales_Report_Audit.xlsx
+++ b/public/downloads/Separate_July_Sales_Report_Audit.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="1" r:id="Ra47dcc3d9ec3460a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Audit" sheetId="2" r:id="Rbc6199b22b614f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Payment Review" sheetId="3" r:id="R0556afe3216c477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Fix Map" sheetId="4" r:id="R3dfba8bd24fc42f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="1" r:id="Rb6c2ec45c2504745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Audit" sheetId="2" r:id="Ra4e0cbd0c3d1404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Payment Review" sheetId="3" r:id="Rb86dbeab10954fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Fix Map" sheetId="4" r:id="R6e2dc74ff92c47a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Colour Legend" sheetId="5" r:id="R336210c3837543c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +20,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0.00;[Red](#,##0.00);-"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,8 +61,32 @@
       <x:color rgb="FFB54708"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF262100"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF211D00"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF063E3A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -78,6 +103,81 @@
         <x:fgColor rgb="FFEAF3EF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7B57A5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3668A9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F9470"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF58220"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFD800"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3F8A5D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF386C9B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF52677D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFDB00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF00CDBC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF36A853"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7C3F98"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA36B12"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB43B35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF68756F"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -85,7 +185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +207,82 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -675,10 +851,10 @@
       <x:c r="C2" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="D2" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E2" t="str">
+      <x:c r="E2" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F2" s="5" t="n">
@@ -724,10 +900,10 @@
       <x:c r="C3" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D3" t="str">
+      <x:c r="D3" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E3" t="str">
+      <x:c r="E3" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F3" s="5" t="n">
@@ -773,10 +949,10 @@
       <x:c r="C4" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D4" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="E4" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F4" s="5" t="n">
@@ -822,10 +998,10 @@
       <x:c r="C5" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="D5" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="E5" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F5" s="5" t="n">
@@ -871,10 +1047,10 @@
       <x:c r="C6" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D6" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E6" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F6" s="5" t="n">
@@ -920,10 +1096,10 @@
       <x:c r="C7" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D7" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E7" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F7" s="5" t="n">
@@ -969,10 +1145,10 @@
       <x:c r="C8" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D8" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="E8" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F8" s="5" t="n">
@@ -1018,10 +1194,10 @@
       <x:c r="C9" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D9" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="E9" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F9" s="5" t="n">
@@ -1067,10 +1243,10 @@
       <x:c r="C10" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F10" s="5" t="n">
@@ -1116,10 +1292,10 @@
       <x:c r="C11" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E11" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F11" s="5" t="n">
@@ -1165,10 +1341,10 @@
       <x:c r="C12" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E12" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F12" s="5" t="n">
@@ -1214,10 +1390,10 @@
       <x:c r="C13" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E13" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F13" s="5" t="n">
@@ -1263,10 +1439,10 @@
       <x:c r="C14" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E14" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F14" s="5" t="n">
@@ -1312,10 +1488,10 @@
       <x:c r="C15" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="E15" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F15" s="5" t="n">
@@ -1361,10 +1537,10 @@
       <x:c r="C16" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E16" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F16" s="5" t="n">
@@ -1410,10 +1586,10 @@
       <x:c r="C17" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D17" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E17" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F17" s="5" t="n">
@@ -1459,10 +1635,10 @@
       <x:c r="C18" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D18" t="str">
+      <x:c r="D18" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="E18" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F18" s="5" t="n">
@@ -1510,10 +1686,10 @@
       <x:c r="C19" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D19" t="str">
+      <x:c r="D19" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E19" t="str">
+      <x:c r="E19" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F19" s="5" t="n">
@@ -1559,10 +1735,10 @@
       <x:c r="C20" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D20" t="str">
+      <x:c r="D20" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E20" t="str">
+      <x:c r="E20" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F20" s="5" t="n">
@@ -1608,10 +1784,10 @@
       <x:c r="C21" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D21" t="str">
+      <x:c r="D21" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E21" t="str">
+      <x:c r="E21" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F21" s="5" t="n">
@@ -1657,7 +1833,7 @@
       <x:c r="C22" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D22" t="str">
+      <x:c r="D22" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E22" t="str">
@@ -1706,10 +1882,10 @@
       <x:c r="C23" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D23" t="str">
+      <x:c r="D23" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E23" t="str">
+      <x:c r="E23" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F23" s="5" t="n">
@@ -1755,10 +1931,10 @@
       <x:c r="C24" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D24" t="str">
+      <x:c r="D24" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E24" t="str">
+      <x:c r="E24" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F24" s="5" t="n">
@@ -1804,7 +1980,7 @@
       <x:c r="C25" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D25" t="str">
+      <x:c r="D25" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E25" t="str">
@@ -1853,10 +2029,10 @@
       <x:c r="C26" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D26" t="str">
+      <x:c r="D26" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E26" t="str">
+      <x:c r="E26" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F26" s="5" t="n">
@@ -1902,7 +2078,7 @@
       <x:c r="C27" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D27" t="str">
+      <x:c r="D27" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E27" t="str">
@@ -1951,10 +2127,10 @@
       <x:c r="C28" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D28" t="str">
+      <x:c r="D28" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E28" t="str">
+      <x:c r="E28" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F28" s="5" t="n">
@@ -2000,10 +2176,10 @@
       <x:c r="C29" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D29" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="E29" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F29" s="5" t="n">
@@ -2049,10 +2225,10 @@
       <x:c r="C30" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D30" t="str">
+      <x:c r="D30" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E30" t="str">
+      <x:c r="E30" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F30" s="5" t="n">
@@ -2098,10 +2274,10 @@
       <x:c r="C31" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D31" t="str">
+      <x:c r="D31" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E31" t="str">
+      <x:c r="E31" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F31" s="5" t="n">
@@ -2147,10 +2323,10 @@
       <x:c r="C32" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D32" t="str">
+      <x:c r="D32" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E32" t="str">
+      <x:c r="E32" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F32" s="5" t="n">
@@ -2196,10 +2372,10 @@
       <x:c r="C33" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D33" t="str">
+      <x:c r="D33" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E33" t="str">
+      <x:c r="E33" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F33" s="5" t="n">
@@ -2245,10 +2421,10 @@
       <x:c r="C34" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D34" t="str">
+      <x:c r="D34" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E34" t="str">
+      <x:c r="E34" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F34" s="5" t="n">
@@ -2294,10 +2470,10 @@
       <x:c r="C35" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D35" t="str">
+      <x:c r="D35" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E35" t="str">
+      <x:c r="E35" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F35" s="5" t="n">
@@ -2343,7 +2519,7 @@
       <x:c r="C36" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D36" t="str">
+      <x:c r="D36" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E36" t="str">
@@ -2392,10 +2568,10 @@
       <x:c r="C37" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D37" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E37" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F37" s="5" t="n">
@@ -2441,10 +2617,10 @@
       <x:c r="C38" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D38" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E38" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F38" s="5" t="n">
@@ -2490,10 +2666,10 @@
       <x:c r="C39" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D39" t="str">
+      <x:c r="D39" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E39" t="str">
+      <x:c r="E39" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F39" s="5" t="n">
@@ -2539,10 +2715,10 @@
       <x:c r="C40" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D40" t="str">
+      <x:c r="D40" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E40" t="str">
+      <x:c r="E40" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F40" s="5" t="n">
@@ -2588,10 +2764,10 @@
       <x:c r="C41" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D41" t="str">
+      <x:c r="D41" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E41" t="str">
+      <x:c r="E41" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F41" s="5" t="n">
@@ -2637,10 +2813,10 @@
       <x:c r="C42" t="str">
         <x:v>20-7-2026</x:v>
       </x:c>
-      <x:c r="D42" t="str">
+      <x:c r="D42" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E42" t="str">
+      <x:c r="E42" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F42" s="5" t="n">
@@ -2686,10 +2862,10 @@
       <x:c r="C43" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D43" t="str">
+      <x:c r="D43" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E43" t="str">
+      <x:c r="E43" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F43" s="5" t="n">
@@ -2735,10 +2911,10 @@
       <x:c r="C44" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D44" t="str">
+      <x:c r="D44" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E44" t="str">
+      <x:c r="E44" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F44" s="5" t="n">
@@ -2784,10 +2960,10 @@
       <x:c r="C45" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D45" t="str">
+      <x:c r="D45" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E45" t="str">
+      <x:c r="E45" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F45" s="5" t="n">
@@ -2833,10 +3009,10 @@
       <x:c r="C46" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D46" t="str">
+      <x:c r="D46" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E46" t="str">
+      <x:c r="E46" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F46" s="5" t="n">
@@ -2882,10 +3058,10 @@
       <x:c r="C47" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D47" t="str">
+      <x:c r="D47" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E47" t="str">
+      <x:c r="E47" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F47" s="5" t="n">
@@ -2931,10 +3107,10 @@
       <x:c r="C48" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D48" t="str">
+      <x:c r="D48" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E48" t="str">
+      <x:c r="E48" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F48" s="5" t="n">
@@ -2980,10 +3156,10 @@
       <x:c r="C49" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D49" t="str">
+      <x:c r="D49" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E49" t="str">
+      <x:c r="E49" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F49" s="5" t="n">
@@ -3029,10 +3205,10 @@
       <x:c r="C50" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D50" t="str">
+      <x:c r="D50" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E50" t="str">
+      <x:c r="E50" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F50" s="5" t="n">
@@ -3078,10 +3254,10 @@
       <x:c r="C51" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D51" t="str">
+      <x:c r="D51" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E51" t="str">
+      <x:c r="E51" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F51" s="5" t="n">
@@ -3129,10 +3305,10 @@
       <x:c r="C52" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D52" t="str">
+      <x:c r="D52" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E52" t="str">
+      <x:c r="E52" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F52" s="5" t="n">
@@ -3180,10 +3356,10 @@
       <x:c r="C53" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D53" t="str">
+      <x:c r="D53" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E53" t="str">
+      <x:c r="E53" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F53" s="5" t="n">
@@ -3229,10 +3405,10 @@
       <x:c r="C54" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D54" t="str">
+      <x:c r="D54" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E54" t="str">
+      <x:c r="E54" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F54" s="5" t="n">
@@ -3278,10 +3454,10 @@
       <x:c r="C55" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D55" t="str">
+      <x:c r="D55" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E55" t="str">
+      <x:c r="E55" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F55" s="5" t="n">
@@ -3327,10 +3503,10 @@
       <x:c r="C56" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D56" t="str">
+      <x:c r="D56" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E56" t="str">
+      <x:c r="E56" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F56" s="5" t="n">
@@ -3378,10 +3554,10 @@
       <x:c r="C57" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D57" t="str">
+      <x:c r="D57" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E57" t="str">
+      <x:c r="E57" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F57" s="5" t="n">
@@ -3429,10 +3605,10 @@
       <x:c r="C58" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D58" t="str">
+      <x:c r="D58" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E58" t="str">
+      <x:c r="E58" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F58" s="5" t="n">
@@ -3478,10 +3654,10 @@
       <x:c r="C59" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D59" t="str">
+      <x:c r="D59" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E59" t="str">
+      <x:c r="E59" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F59" s="5" t="n">
@@ -3527,10 +3703,10 @@
       <x:c r="C60" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D60" t="str">
+      <x:c r="D60" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E60" t="str">
+      <x:c r="E60" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F60" s="5" t="n">
@@ -3578,10 +3754,10 @@
       <x:c r="C61" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D61" t="str">
+      <x:c r="D61" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E61" t="str">
+      <x:c r="E61" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F61" s="5" t="n">
@@ -3627,7 +3803,7 @@
       <x:c r="C62" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D62" t="str">
+      <x:c r="D62" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E62" t="str">
@@ -3676,10 +3852,10 @@
       <x:c r="C63" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D63" t="str">
+      <x:c r="D63" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E63" t="str">
+      <x:c r="E63" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F63" s="5" t="n">
@@ -3725,10 +3901,10 @@
       <x:c r="C64" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D64" t="str">
+      <x:c r="D64" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E64" t="str">
+      <x:c r="E64" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F64" s="5" t="n">
@@ -3774,10 +3950,10 @@
       <x:c r="C65" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D65" t="str">
+      <x:c r="D65" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E65" t="str">
+      <x:c r="E65" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F65" s="5" t="n">
@@ -3823,10 +3999,10 @@
       <x:c r="C66" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D66" t="str">
+      <x:c r="D66" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E66" t="str">
+      <x:c r="E66" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F66" s="5" t="n">
@@ -3872,10 +4048,10 @@
       <x:c r="C67" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D67" t="str">
+      <x:c r="D67" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E67" t="str">
+      <x:c r="E67" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F67" s="5" t="n">
@@ -3921,10 +4097,10 @@
       <x:c r="C68" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D68" t="str">
+      <x:c r="D68" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E68" t="str">
+      <x:c r="E68" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F68" s="5" t="n">
@@ -3970,10 +4146,10 @@
       <x:c r="C69" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D69" t="str">
+      <x:c r="D69" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E69" t="str">
+      <x:c r="E69" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F69" s="5" t="n">
@@ -4019,10 +4195,10 @@
       <x:c r="C70" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D70" t="str">
+      <x:c r="D70" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E70" t="str">
+      <x:c r="E70" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F70" s="5" t="n">
@@ -4068,10 +4244,10 @@
       <x:c r="C71" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D71" t="str">
+      <x:c r="D71" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E71" t="str">
+      <x:c r="E71" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F71" s="5" t="n">
@@ -4119,7 +4295,7 @@
       <x:c r="C72" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D72" t="str">
+      <x:c r="D72" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E72" t="str">
@@ -4168,10 +4344,10 @@
       <x:c r="C73" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D73" t="str">
+      <x:c r="D73" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E73" t="str">
+      <x:c r="E73" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F73" s="5" t="n">
@@ -4217,10 +4393,10 @@
       <x:c r="C74" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D74" t="str">
+      <x:c r="D74" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E74" t="str">
+      <x:c r="E74" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F74" s="5" t="n">
@@ -4266,10 +4442,10 @@
       <x:c r="C75" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D75" t="str">
+      <x:c r="D75" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E75" t="str">
+      <x:c r="E75" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F75" s="5" t="n">
@@ -4315,10 +4491,10 @@
       <x:c r="C76" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D76" t="str">
+      <x:c r="D76" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E76" t="str">
+      <x:c r="E76" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F76" s="5" t="n">
@@ -4364,10 +4540,10 @@
       <x:c r="C77" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D77" t="str">
+      <x:c r="D77" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E77" t="str">
+      <x:c r="E77" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F77" s="5" t="n">
@@ -4413,7 +4589,7 @@
       <x:c r="C78" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D78" t="str">
+      <x:c r="D78" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E78" t="str">
@@ -4462,10 +4638,10 @@
       <x:c r="C79" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D79" t="str">
+      <x:c r="D79" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E79" t="str">
+      <x:c r="E79" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F79" s="5" t="n">
@@ -4511,10 +4687,10 @@
       <x:c r="C80" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D80" t="str">
+      <x:c r="D80" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E80" t="str">
+      <x:c r="E80" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F80" s="5" t="n">
@@ -4560,10 +4736,10 @@
       <x:c r="C81" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D81" t="str">
+      <x:c r="D81" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E81" t="str">
+      <x:c r="E81" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F81" s="5" t="n">
@@ -4609,10 +4785,10 @@
       <x:c r="C82" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D82" t="str">
+      <x:c r="D82" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E82" t="str">
+      <x:c r="E82" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F82" s="5" t="n">
@@ -4658,10 +4834,10 @@
       <x:c r="C83" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D83" t="str">
+      <x:c r="D83" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E83" t="str">
+      <x:c r="E83" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F83" s="5" t="n">
@@ -4707,10 +4883,10 @@
       <x:c r="C84" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D84" t="str">
+      <x:c r="D84" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E84" t="str">
+      <x:c r="E84" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F84" s="5" t="n">
@@ -4756,10 +4932,10 @@
       <x:c r="C85" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D85" t="str">
+      <x:c r="D85" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E85" t="str">
+      <x:c r="E85" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F85" s="5" t="n">
@@ -4805,7 +4981,7 @@
       <x:c r="C86" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D86" t="str">
+      <x:c r="D86" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E86" t="str">
@@ -4854,10 +5030,10 @@
       <x:c r="C87" t="str">
         <x:v>21-7-2026</x:v>
       </x:c>
-      <x:c r="D87" t="str">
+      <x:c r="D87" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E87" t="str">
+      <x:c r="E87" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F87" s="5" t="n">
@@ -4903,10 +5079,10 @@
       <x:c r="C88" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D88" t="str">
+      <x:c r="D88" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E88" t="str">
+      <x:c r="E88" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F88" s="5" t="n">
@@ -4952,10 +5128,10 @@
       <x:c r="C89" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D89" t="str">
+      <x:c r="D89" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E89" t="str">
+      <x:c r="E89" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F89" s="5" t="n">
@@ -5001,7 +5177,7 @@
       <x:c r="C90" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D90" t="str">
+      <x:c r="D90" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E90" t="str">
@@ -5050,10 +5226,10 @@
       <x:c r="C91" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D91" t="str">
+      <x:c r="D91" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E91" t="str">
+      <x:c r="E91" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F91" s="5" t="n">
@@ -5099,10 +5275,10 @@
       <x:c r="C92" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D92" t="str">
+      <x:c r="D92" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E92" t="str">
+      <x:c r="E92" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F92" s="5" t="n">
@@ -5150,10 +5326,10 @@
       <x:c r="C93" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D93" t="str">
+      <x:c r="D93" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E93" t="str">
+      <x:c r="E93" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F93" s="5" t="n">
@@ -5199,7 +5375,7 @@
       <x:c r="C94" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D94" t="str">
+      <x:c r="D94" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E94" t="str">
@@ -5250,7 +5426,7 @@
       <x:c r="C95" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D95" t="str">
+      <x:c r="D95" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E95" t="str">
@@ -5299,10 +5475,10 @@
       <x:c r="C96" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D96" t="str">
+      <x:c r="D96" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E96" t="str">
+      <x:c r="E96" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F96" s="5" t="n">
@@ -5348,10 +5524,10 @@
       <x:c r="C97" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D97" t="str">
+      <x:c r="D97" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E97" t="str">
+      <x:c r="E97" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F97" s="5" t="n">
@@ -5397,7 +5573,7 @@
       <x:c r="C98" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D98" t="str">
+      <x:c r="D98" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E98" t="str">
@@ -5446,10 +5622,10 @@
       <x:c r="C99" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D99" t="str">
+      <x:c r="D99" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E99" t="str">
+      <x:c r="E99" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F99" s="5" t="n">
@@ -5495,10 +5671,10 @@
       <x:c r="C100" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D100" t="str">
+      <x:c r="D100" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E100" t="str">
+      <x:c r="E100" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F100" s="5" t="n">
@@ -5544,10 +5720,10 @@
       <x:c r="C101" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D101" t="str">
+      <x:c r="D101" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E101" t="str">
+      <x:c r="E101" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F101" s="5" t="n">
@@ -5593,7 +5769,7 @@
       <x:c r="C102" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D102" t="str">
+      <x:c r="D102" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E102" t="str">
@@ -5642,7 +5818,7 @@
       <x:c r="C103" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D103" t="str">
+      <x:c r="D103" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E103" t="str">
@@ -5691,7 +5867,7 @@
       <x:c r="C104" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D104" t="str">
+      <x:c r="D104" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E104" t="str">
@@ -5740,10 +5916,10 @@
       <x:c r="C105" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D105" t="str">
+      <x:c r="D105" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E105" t="str">
+      <x:c r="E105" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F105" s="5" t="n">
@@ -5789,7 +5965,7 @@
       <x:c r="C106" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D106" t="str">
+      <x:c r="D106" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E106" t="str">
@@ -5838,10 +6014,10 @@
       <x:c r="C107" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D107" t="str">
+      <x:c r="D107" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E107" t="str">
+      <x:c r="E107" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F107" s="5" t="n">
@@ -5887,10 +6063,10 @@
       <x:c r="C108" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D108" t="str">
+      <x:c r="D108" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E108" t="str">
+      <x:c r="E108" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F108" s="5" t="n">
@@ -5936,10 +6112,10 @@
       <x:c r="C109" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D109" t="str">
+      <x:c r="D109" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E109" t="str">
+      <x:c r="E109" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F109" s="5" t="n">
@@ -5985,7 +6161,7 @@
       <x:c r="C110" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D110" t="str">
+      <x:c r="D110" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E110" t="str">
@@ -6034,10 +6210,10 @@
       <x:c r="C111" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D111" t="str">
+      <x:c r="D111" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E111" t="str">
+      <x:c r="E111" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F111" s="5" t="n">
@@ -6083,10 +6259,10 @@
       <x:c r="C112" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D112" t="str">
+      <x:c r="D112" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E112" t="str">
+      <x:c r="E112" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F112" s="5" t="n">
@@ -6132,7 +6308,7 @@
       <x:c r="C113" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D113" t="str">
+      <x:c r="D113" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E113" t="str">
@@ -6181,10 +6357,10 @@
       <x:c r="C114" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D114" t="str">
+      <x:c r="D114" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E114" t="str">
+      <x:c r="E114" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F114" s="5" t="n">
@@ -6230,10 +6406,10 @@
       <x:c r="C115" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D115" t="str">
+      <x:c r="D115" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E115" t="str">
+      <x:c r="E115" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F115" s="5" t="n">
@@ -6281,10 +6457,10 @@
       <x:c r="C116" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D116" t="str">
+      <x:c r="D116" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E116" t="str">
+      <x:c r="E116" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F116" s="5" t="n">
@@ -6330,7 +6506,7 @@
       <x:c r="C117" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D117" t="str">
+      <x:c r="D117" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E117" t="str">
@@ -6379,7 +6555,7 @@
       <x:c r="C118" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D118" t="str">
+      <x:c r="D118" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E118" t="str">
@@ -6428,7 +6604,7 @@
       <x:c r="C119" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D119" t="str">
+      <x:c r="D119" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E119" t="str">
@@ -6477,7 +6653,7 @@
       <x:c r="C120" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D120" t="str">
+      <x:c r="D120" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E120" t="str">
@@ -6526,7 +6702,7 @@
       <x:c r="C121" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D121" t="str">
+      <x:c r="D121" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E121" t="str">
@@ -6575,7 +6751,7 @@
       <x:c r="C122" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D122" t="str">
+      <x:c r="D122" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E122" t="str">
@@ -6624,10 +6800,10 @@
       <x:c r="C123" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D123" t="str">
+      <x:c r="D123" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E123" t="str">
+      <x:c r="E123" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F123" s="5" t="n">
@@ -6673,10 +6849,10 @@
       <x:c r="C124" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D124" t="str">
+      <x:c r="D124" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E124" t="str">
+      <x:c r="E124" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F124" s="5" t="n">
@@ -6722,7 +6898,7 @@
       <x:c r="C125" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D125" t="str">
+      <x:c r="D125" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E125" t="str">
@@ -6771,7 +6947,7 @@
       <x:c r="C126" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D126" t="str">
+      <x:c r="D126" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E126" t="str">
@@ -6820,10 +6996,10 @@
       <x:c r="C127" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D127" t="str">
+      <x:c r="D127" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E127" t="str">
+      <x:c r="E127" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F127" s="5" t="n">
@@ -6869,10 +7045,10 @@
       <x:c r="C128" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D128" t="str">
+      <x:c r="D128" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E128" t="str">
+      <x:c r="E128" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F128" s="5" t="n">
@@ -6918,7 +7094,7 @@
       <x:c r="C129" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D129" t="str">
+      <x:c r="D129" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E129" t="str">
@@ -6967,7 +7143,7 @@
       <x:c r="C130" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D130" t="str">
+      <x:c r="D130" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E130" t="str">
@@ -7016,7 +7192,7 @@
       <x:c r="C131" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D131" t="str">
+      <x:c r="D131" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E131" t="str">
@@ -7065,10 +7241,10 @@
       <x:c r="C132" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D132" t="str">
+      <x:c r="D132" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E132" t="str">
+      <x:c r="E132" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F132" s="5" t="n">
@@ -7114,7 +7290,7 @@
       <x:c r="C133" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D133" t="str">
+      <x:c r="D133" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E133" t="str">
@@ -7163,7 +7339,7 @@
       <x:c r="C134" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D134" t="str">
+      <x:c r="D134" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
       <x:c r="E134" t="str">
@@ -7212,7 +7388,7 @@
       <x:c r="C135" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D135" t="str">
+      <x:c r="D135" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E135" t="str">
@@ -7261,10 +7437,10 @@
       <x:c r="C136" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D136" t="str">
+      <x:c r="D136" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E136" t="str">
+      <x:c r="E136" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F136" s="5" t="n">
@@ -7310,7 +7486,7 @@
       <x:c r="C137" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D137" t="str">
+      <x:c r="D137" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E137" t="str">
@@ -7359,10 +7535,10 @@
       <x:c r="C138" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D138" t="str">
+      <x:c r="D138" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E138" t="str">
+      <x:c r="E138" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F138" s="5" t="n">
@@ -7408,10 +7584,10 @@
       <x:c r="C139" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D139" t="str">
+      <x:c r="D139" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E139" t="str">
+      <x:c r="E139" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F139" s="5" t="n">
@@ -7457,7 +7633,7 @@
       <x:c r="C140" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D140" t="str">
+      <x:c r="D140" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E140" t="str">
@@ -7506,10 +7682,10 @@
       <x:c r="C141" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D141" t="str">
+      <x:c r="D141" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E141" t="str">
+      <x:c r="E141" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F141" s="5" t="n">
@@ -7555,7 +7731,7 @@
       <x:c r="C142" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D142" t="str">
+      <x:c r="D142" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E142" t="str">
@@ -7604,10 +7780,10 @@
       <x:c r="C143" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D143" t="str">
+      <x:c r="D143" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E143" t="str">
+      <x:c r="E143" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F143" s="5" t="n">
@@ -7653,10 +7829,10 @@
       <x:c r="C144" t="str">
         <x:v>22-7-2026</x:v>
       </x:c>
-      <x:c r="D144" t="str">
+      <x:c r="D144" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E144" t="str">
+      <x:c r="E144" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F144" s="5" t="n">
@@ -7702,10 +7878,10 @@
       <x:c r="C145" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D145" t="str">
+      <x:c r="D145" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E145" t="str">
+      <x:c r="E145" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F145" s="5" t="n">
@@ -7751,10 +7927,10 @@
       <x:c r="C146" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D146" t="str">
+      <x:c r="D146" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E146" t="str">
+      <x:c r="E146" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F146" s="5" t="n">
@@ -7800,7 +7976,7 @@
       <x:c r="C147" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D147" t="str">
+      <x:c r="D147" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E147" t="str">
@@ -7849,10 +8025,10 @@
       <x:c r="C148" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D148" t="str">
+      <x:c r="D148" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E148" t="str">
+      <x:c r="E148" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F148" s="5" t="n">
@@ -7898,10 +8074,10 @@
       <x:c r="C149" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D149" t="str">
+      <x:c r="D149" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E149" t="str">
+      <x:c r="E149" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F149" s="5" t="n">
@@ -7947,10 +8123,10 @@
       <x:c r="C150" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D150" t="str">
+      <x:c r="D150" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E150" t="str">
+      <x:c r="E150" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F150" s="5" t="n">
@@ -7996,10 +8172,10 @@
       <x:c r="C151" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D151" t="str">
+      <x:c r="D151" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E151" t="str">
+      <x:c r="E151" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F151" s="5" t="n">
@@ -8045,10 +8221,10 @@
       <x:c r="C152" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D152" t="str">
+      <x:c r="D152" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E152" t="str">
+      <x:c r="E152" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F152" s="5" t="n">
@@ -8094,7 +8270,7 @@
       <x:c r="C153" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D153" t="str">
+      <x:c r="D153" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E153" t="str">
@@ -8143,10 +8319,10 @@
       <x:c r="C154" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D154" t="str">
+      <x:c r="D154" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E154" t="str">
+      <x:c r="E154" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F154" s="5" t="n">
@@ -8192,10 +8368,10 @@
       <x:c r="C155" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D155" t="str">
+      <x:c r="D155" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E155" t="str">
+      <x:c r="E155" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F155" s="5" t="n">
@@ -8241,10 +8417,10 @@
       <x:c r="C156" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D156" t="str">
+      <x:c r="D156" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E156" t="str">
+      <x:c r="E156" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F156" s="5" t="n">
@@ -8290,10 +8466,10 @@
       <x:c r="C157" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D157" t="str">
+      <x:c r="D157" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E157" t="str">
+      <x:c r="E157" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F157" s="5" t="n">
@@ -8339,7 +8515,7 @@
       <x:c r="C158" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D158" t="str">
+      <x:c r="D158" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E158" t="str">
@@ -8388,10 +8564,10 @@
       <x:c r="C159" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D159" t="str">
+      <x:c r="D159" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E159" t="str">
+      <x:c r="E159" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F159" s="5" t="n">
@@ -8437,10 +8613,10 @@
       <x:c r="C160" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D160" t="str">
+      <x:c r="D160" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E160" t="str">
+      <x:c r="E160" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F160" s="5" t="n">
@@ -8486,10 +8662,10 @@
       <x:c r="C161" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D161" t="str">
+      <x:c r="D161" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E161" t="str">
+      <x:c r="E161" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F161" s="5" t="n">
@@ -8535,10 +8711,10 @@
       <x:c r="C162" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D162" t="str">
+      <x:c r="D162" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E162" t="str">
+      <x:c r="E162" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F162" s="5" t="n">
@@ -8584,10 +8760,10 @@
       <x:c r="C163" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D163" t="str">
+      <x:c r="D163" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E163" t="str">
+      <x:c r="E163" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F163" s="5" t="n">
@@ -8633,10 +8809,10 @@
       <x:c r="C164" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D164" t="str">
+      <x:c r="D164" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E164" t="str">
+      <x:c r="E164" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F164" s="5" t="n">
@@ -8682,10 +8858,10 @@
       <x:c r="C165" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D165" t="str">
+      <x:c r="D165" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E165" t="str">
+      <x:c r="E165" s="35" t="str">
         <x:v>Card,Cash</x:v>
       </x:c>
       <x:c r="F165" s="5" t="n">
@@ -8733,10 +8909,10 @@
       <x:c r="C166" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D166" t="str">
+      <x:c r="D166" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E166" t="str">
+      <x:c r="E166" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F166" s="5" t="n">
@@ -8782,10 +8958,10 @@
       <x:c r="C167" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D167" t="str">
+      <x:c r="D167" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E167" t="str">
+      <x:c r="E167" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F167" s="5" t="n">
@@ -8831,7 +9007,7 @@
       <x:c r="C168" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D168" t="str">
+      <x:c r="D168" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E168" t="str">
@@ -8880,10 +9056,10 @@
       <x:c r="C169" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D169" t="str">
+      <x:c r="D169" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E169" t="str">
+      <x:c r="E169" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F169" s="5" t="n">
@@ -8929,10 +9105,10 @@
       <x:c r="C170" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D170" t="str">
+      <x:c r="D170" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E170" t="str">
+      <x:c r="E170" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F170" s="5" t="n">
@@ -8978,10 +9154,10 @@
       <x:c r="C171" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D171" t="str">
+      <x:c r="D171" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E171" t="str">
+      <x:c r="E171" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F171" s="5" t="n">
@@ -9027,10 +9203,10 @@
       <x:c r="C172" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D172" t="str">
+      <x:c r="D172" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E172" t="str">
+      <x:c r="E172" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F172" s="5" t="n">
@@ -9076,7 +9252,7 @@
       <x:c r="C173" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D173" t="str">
+      <x:c r="D173" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E173" t="str">
@@ -9125,10 +9301,10 @@
       <x:c r="C174" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D174" t="str">
+      <x:c r="D174" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E174" t="str">
+      <x:c r="E174" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F174" s="5" t="n">
@@ -9174,10 +9350,10 @@
       <x:c r="C175" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D175" t="str">
+      <x:c r="D175" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E175" t="str">
+      <x:c r="E175" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F175" s="5" t="n">
@@ -9223,10 +9399,10 @@
       <x:c r="C176" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D176" t="str">
+      <x:c r="D176" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E176" t="str">
+      <x:c r="E176" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F176" s="5" t="n">
@@ -9272,10 +9448,10 @@
       <x:c r="C177" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D177" t="str">
+      <x:c r="D177" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E177" t="str">
+      <x:c r="E177" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F177" s="5" t="n">
@@ -9321,10 +9497,10 @@
       <x:c r="C178" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D178" t="str">
+      <x:c r="D178" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E178" t="str">
+      <x:c r="E178" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F178" s="5" t="n">
@@ -9370,10 +9546,10 @@
       <x:c r="C179" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D179" t="str">
+      <x:c r="D179" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E179" t="str">
+      <x:c r="E179" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F179" s="5" t="n">
@@ -9419,10 +9595,10 @@
       <x:c r="C180" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D180" t="str">
+      <x:c r="D180" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E180" t="str">
+      <x:c r="E180" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F180" s="5" t="n">
@@ -9468,10 +9644,10 @@
       <x:c r="C181" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D181" t="str">
+      <x:c r="D181" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E181" t="str">
+      <x:c r="E181" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F181" s="5" t="n">
@@ -9517,10 +9693,10 @@
       <x:c r="C182" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D182" t="str">
+      <x:c r="D182" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E182" t="str">
+      <x:c r="E182" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F182" s="5" t="n">
@@ -9566,10 +9742,10 @@
       <x:c r="C183" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D183" t="str">
+      <x:c r="D183" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E183" t="str">
+      <x:c r="E183" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F183" s="5" t="n">
@@ -9615,10 +9791,10 @@
       <x:c r="C184" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D184" t="str">
+      <x:c r="D184" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E184" t="str">
+      <x:c r="E184" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F184" s="5" t="n">
@@ -9664,10 +9840,10 @@
       <x:c r="C185" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D185" t="str">
+      <x:c r="D185" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E185" t="str">
+      <x:c r="E185" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F185" s="5" t="n">
@@ -9713,10 +9889,10 @@
       <x:c r="C186" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D186" t="str">
+      <x:c r="D186" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E186" t="str">
+      <x:c r="E186" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F186" s="5" t="n">
@@ -9762,10 +9938,10 @@
       <x:c r="C187" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D187" t="str">
+      <x:c r="D187" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E187" t="str">
+      <x:c r="E187" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F187" s="5" t="n">
@@ -9811,10 +9987,10 @@
       <x:c r="C188" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D188" t="str">
+      <x:c r="D188" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E188" t="str">
+      <x:c r="E188" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F188" s="5" t="n">
@@ -9860,7 +10036,7 @@
       <x:c r="C189" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D189" t="str">
+      <x:c r="D189" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E189" t="str">
@@ -9909,10 +10085,10 @@
       <x:c r="C190" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D190" t="str">
+      <x:c r="D190" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E190" t="str">
+      <x:c r="E190" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F190" s="5" t="n">
@@ -9958,7 +10134,7 @@
       <x:c r="C191" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D191" t="str">
+      <x:c r="D191" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E191" t="str">
@@ -10007,10 +10183,10 @@
       <x:c r="C192" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D192" t="str">
+      <x:c r="D192" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
-      <x:c r="E192" t="str">
+      <x:c r="E192" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F192" s="5" t="n">
@@ -10056,10 +10232,10 @@
       <x:c r="C193" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D193" t="str">
+      <x:c r="D193" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E193" t="str">
+      <x:c r="E193" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F193" s="5" t="n">
@@ -10105,10 +10281,10 @@
       <x:c r="C194" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D194" t="str">
+      <x:c r="D194" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
-      <x:c r="E194" t="str">
+      <x:c r="E194" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F194" s="5" t="n">
@@ -10154,10 +10330,10 @@
       <x:c r="C195" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D195" t="str">
+      <x:c r="D195" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E195" t="str">
+      <x:c r="E195" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F195" s="5" t="n">
@@ -10203,10 +10379,10 @@
       <x:c r="C196" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D196" t="str">
+      <x:c r="D196" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E196" t="str">
+      <x:c r="E196" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F196" s="5" t="n">
@@ -10252,10 +10428,10 @@
       <x:c r="C197" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D197" t="str">
+      <x:c r="D197" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E197" t="str">
+      <x:c r="E197" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F197" s="5" t="n">
@@ -10301,10 +10477,10 @@
       <x:c r="C198" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D198" t="str">
+      <x:c r="D198" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E198" t="str">
+      <x:c r="E198" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F198" s="5" t="n">
@@ -10350,10 +10526,10 @@
       <x:c r="C199" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D199" t="str">
+      <x:c r="D199" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E199" t="str">
+      <x:c r="E199" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F199" s="5" t="n">
@@ -10399,10 +10575,10 @@
       <x:c r="C200" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E200" t="str">
+      <x:c r="E200" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F200" s="5" t="n">
@@ -10448,10 +10624,10 @@
       <x:c r="C201" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E201" t="str">
+      <x:c r="E201" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F201" s="5" t="n">
@@ -10497,10 +10673,10 @@
       <x:c r="C202" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D202" t="str">
+      <x:c r="D202" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E202" t="str">
+      <x:c r="E202" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F202" s="5" t="n">
@@ -10546,7 +10722,7 @@
       <x:c r="C203" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D203" t="str">
+      <x:c r="D203" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E203" t="str">
@@ -10595,10 +10771,10 @@
       <x:c r="C204" t="str">
         <x:v>23-7-2026</x:v>
       </x:c>
-      <x:c r="D204" t="str">
+      <x:c r="D204" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E204" t="str">
+      <x:c r="E204" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F204" s="5" t="n">
@@ -10644,10 +10820,10 @@
       <x:c r="C205" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D205" t="str">
+      <x:c r="D205" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E205" t="str">
+      <x:c r="E205" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F205" s="5" t="n">
@@ -10693,10 +10869,10 @@
       <x:c r="C206" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D206" t="str">
+      <x:c r="D206" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E206" t="str">
+      <x:c r="E206" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F206" s="5" t="n">
@@ -10742,10 +10918,10 @@
       <x:c r="C207" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D207" t="str">
+      <x:c r="D207" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E207" t="str">
+      <x:c r="E207" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F207" s="5" t="n">
@@ -10791,7 +10967,7 @@
       <x:c r="C208" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D208" t="str">
+      <x:c r="D208" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E208" t="str">
@@ -10840,10 +11016,10 @@
       <x:c r="C209" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D209" t="str">
+      <x:c r="D209" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E209" t="str">
+      <x:c r="E209" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F209" s="5" t="n">
@@ -10889,10 +11065,10 @@
       <x:c r="C210" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D210" t="str">
+      <x:c r="D210" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E210" t="str">
+      <x:c r="E210" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F210" s="5" t="n">
@@ -10938,10 +11114,10 @@
       <x:c r="C211" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D211" t="str">
+      <x:c r="D211" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E211" t="str">
+      <x:c r="E211" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F211" s="5" t="n">
@@ -10987,10 +11163,10 @@
       <x:c r="C212" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D212" t="str">
+      <x:c r="D212" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E212" t="str">
+      <x:c r="E212" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F212" s="5" t="n">
@@ -11036,10 +11212,10 @@
       <x:c r="C213" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D213" t="str">
+      <x:c r="D213" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E213" t="str">
+      <x:c r="E213" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F213" s="5" t="n">
@@ -11085,10 +11261,10 @@
       <x:c r="C214" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D214" t="str">
+      <x:c r="D214" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E214" t="str">
+      <x:c r="E214" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F214" s="5" t="n">
@@ -11134,10 +11310,10 @@
       <x:c r="C215" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D215" t="str">
+      <x:c r="D215" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E215" t="str">
+      <x:c r="E215" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F215" s="5" t="n">
@@ -11183,10 +11359,10 @@
       <x:c r="C216" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D216" t="str">
+      <x:c r="D216" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E216" t="str">
+      <x:c r="E216" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F216" s="5" t="n">
@@ -11234,10 +11410,10 @@
       <x:c r="C217" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D217" t="str">
+      <x:c r="D217" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E217" t="str">
+      <x:c r="E217" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F217" s="5" t="n">
@@ -11283,7 +11459,7 @@
       <x:c r="C218" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D218" t="str">
+      <x:c r="D218" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E218" t="str">
@@ -11332,10 +11508,10 @@
       <x:c r="C219" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D219" t="str">
+      <x:c r="D219" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E219" t="str">
+      <x:c r="E219" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F219" s="5" t="n">
@@ -11383,10 +11559,10 @@
       <x:c r="C220" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D220" t="str">
+      <x:c r="D220" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E220" t="str">
+      <x:c r="E220" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F220" s="5" t="n">
@@ -11434,10 +11610,10 @@
       <x:c r="C221" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D221" t="str">
+      <x:c r="D221" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E221" t="str">
+      <x:c r="E221" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F221" s="5" t="n">
@@ -11483,7 +11659,7 @@
       <x:c r="C222" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D222" t="str">
+      <x:c r="D222" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E222" t="str">
@@ -11532,7 +11708,7 @@
       <x:c r="C223" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D223" t="str">
+      <x:c r="D223" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E223" t="str">
@@ -11581,10 +11757,10 @@
       <x:c r="C224" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D224" t="str">
+      <x:c r="D224" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E224" t="str">
+      <x:c r="E224" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F224" s="5" t="n">
@@ -11630,10 +11806,10 @@
       <x:c r="C225" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D225" t="str">
+      <x:c r="D225" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E225" t="str">
+      <x:c r="E225" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F225" s="5" t="n">
@@ -11679,10 +11855,10 @@
       <x:c r="C226" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D226" t="str">
+      <x:c r="D226" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E226" t="str">
+      <x:c r="E226" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F226" s="5" t="n">
@@ -11728,10 +11904,10 @@
       <x:c r="C227" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D227" t="str">
+      <x:c r="D227" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E227" t="str">
+      <x:c r="E227" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F227" s="5" t="n">
@@ -11777,10 +11953,10 @@
       <x:c r="C228" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D228" t="str">
+      <x:c r="D228" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E228" t="str">
+      <x:c r="E228" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F228" s="5" t="n">
@@ -11826,10 +12002,10 @@
       <x:c r="C229" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D229" t="str">
+      <x:c r="D229" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E229" t="str">
+      <x:c r="E229" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F229" s="5" t="n">
@@ -11875,10 +12051,10 @@
       <x:c r="C230" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D230" t="str">
+      <x:c r="D230" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E230" t="str">
+      <x:c r="E230" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F230" s="5" t="n">
@@ -11924,10 +12100,10 @@
       <x:c r="C231" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D231" t="str">
+      <x:c r="D231" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E231" t="str">
+      <x:c r="E231" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F231" s="5" t="n">
@@ -11973,10 +12149,10 @@
       <x:c r="C232" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D232" t="str">
+      <x:c r="D232" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E232" t="str">
+      <x:c r="E232" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F232" s="5" t="n">
@@ -12022,10 +12198,10 @@
       <x:c r="C233" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D233" t="str">
+      <x:c r="D233" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E233" t="str">
+      <x:c r="E233" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F233" s="5" t="n">
@@ -12071,10 +12247,10 @@
       <x:c r="C234" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D234" t="str">
+      <x:c r="D234" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E234" t="str">
+      <x:c r="E234" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F234" s="5" t="n">
@@ -12120,10 +12296,10 @@
       <x:c r="C235" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D235" t="str">
+      <x:c r="D235" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E235" t="str">
+      <x:c r="E235" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F235" s="5" t="n">
@@ -12169,10 +12345,10 @@
       <x:c r="C236" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D236" t="str">
+      <x:c r="D236" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E236" t="str">
+      <x:c r="E236" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F236" s="5" t="n">
@@ -12218,10 +12394,10 @@
       <x:c r="C237" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D237" t="str">
+      <x:c r="D237" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E237" t="str">
+      <x:c r="E237" s="35" t="str">
         <x:v>Card,Cash</x:v>
       </x:c>
       <x:c r="F237" s="5" t="n">
@@ -12269,10 +12445,10 @@
       <x:c r="C238" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D238" t="str">
+      <x:c r="D238" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
-      <x:c r="E238" t="str">
+      <x:c r="E238" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F238" s="5" t="n">
@@ -12318,10 +12494,10 @@
       <x:c r="C239" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D239" t="str">
+      <x:c r="D239" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E239" t="str">
+      <x:c r="E239" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F239" s="5" t="n">
@@ -12367,10 +12543,10 @@
       <x:c r="C240" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D240" t="str">
+      <x:c r="D240" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E240" t="str">
+      <x:c r="E240" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F240" s="5" t="n">
@@ -12416,10 +12592,10 @@
       <x:c r="C241" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D241" t="str">
+      <x:c r="D241" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E241" t="str">
+      <x:c r="E241" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F241" s="5" t="n">
@@ -12465,10 +12641,10 @@
       <x:c r="C242" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D242" t="str">
+      <x:c r="D242" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E242" t="str">
+      <x:c r="E242" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F242" s="5" t="n">
@@ -12514,10 +12690,10 @@
       <x:c r="C243" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D243" t="str">
+      <x:c r="D243" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E243" t="str">
+      <x:c r="E243" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F243" s="5" t="n">
@@ -12563,10 +12739,10 @@
       <x:c r="C244" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D244" t="str">
+      <x:c r="D244" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E244" t="str">
+      <x:c r="E244" s="35" t="str">
         <x:v>Card,Cash</x:v>
       </x:c>
       <x:c r="F244" s="5" t="n">
@@ -12614,10 +12790,10 @@
       <x:c r="C245" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D245" t="str">
+      <x:c r="D245" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E245" t="str">
+      <x:c r="E245" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F245" s="5" t="n">
@@ -12663,10 +12839,10 @@
       <x:c r="C246" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D246" t="str">
+      <x:c r="D246" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E246" t="str">
+      <x:c r="E246" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F246" s="5" t="n">
@@ -12712,10 +12888,10 @@
       <x:c r="C247" t="str">
         <x:v>24-7-2026</x:v>
       </x:c>
-      <x:c r="D247" t="str">
+      <x:c r="D247" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E247" t="str">
+      <x:c r="E247" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F247" s="5" t="n">
@@ -12761,10 +12937,10 @@
       <x:c r="C248" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D248" t="str">
+      <x:c r="D248" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E248" t="str">
+      <x:c r="E248" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F248" s="5" t="n">
@@ -12810,10 +12986,10 @@
       <x:c r="C249" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D249" t="str">
+      <x:c r="D249" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E249" t="str">
+      <x:c r="E249" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F249" s="5" t="n">
@@ -12859,7 +13035,7 @@
       <x:c r="C250" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D250" t="str">
+      <x:c r="D250" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E250" t="str">
@@ -12908,7 +13084,7 @@
       <x:c r="C251" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D251" t="str">
+      <x:c r="D251" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E251" t="str">
@@ -12957,10 +13133,10 @@
       <x:c r="C252" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D252" t="str">
+      <x:c r="D252" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E252" t="str">
+      <x:c r="E252" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F252" s="5" t="n">
@@ -13006,10 +13182,10 @@
       <x:c r="C253" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D253" t="str">
+      <x:c r="D253" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E253" t="str">
+      <x:c r="E253" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F253" s="5" t="n">
@@ -13055,7 +13231,7 @@
       <x:c r="C254" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D254" t="str">
+      <x:c r="D254" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E254" t="str">
@@ -13104,10 +13280,10 @@
       <x:c r="C255" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D255" t="str">
+      <x:c r="D255" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E255" t="str">
+      <x:c r="E255" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F255" s="5" t="n">
@@ -13153,10 +13329,10 @@
       <x:c r="C256" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D256" t="str">
+      <x:c r="D256" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E256" t="str">
+      <x:c r="E256" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F256" s="5" t="n">
@@ -13202,10 +13378,10 @@
       <x:c r="C257" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D257" t="str">
+      <x:c r="D257" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E257" t="str">
+      <x:c r="E257" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F257" s="5" t="n">
@@ -13251,10 +13427,10 @@
       <x:c r="C258" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D258" t="str">
+      <x:c r="D258" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E258" t="str">
+      <x:c r="E258" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F258" s="5" t="n">
@@ -13300,10 +13476,10 @@
       <x:c r="C259" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D259" t="str">
+      <x:c r="D259" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E259" t="str">
+      <x:c r="E259" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F259" s="5" t="n">
@@ -13349,10 +13525,10 @@
       <x:c r="C260" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D260" t="str">
+      <x:c r="D260" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E260" t="str">
+      <x:c r="E260" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F260" s="5" t="n">
@@ -13398,7 +13574,7 @@
       <x:c r="C261" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D261" t="str">
+      <x:c r="D261" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E261" t="str">
@@ -13447,10 +13623,10 @@
       <x:c r="C262" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D262" t="str">
+      <x:c r="D262" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E262" t="str">
+      <x:c r="E262" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F262" s="5" t="n">
@@ -13496,10 +13672,10 @@
       <x:c r="C263" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D263" t="str">
+      <x:c r="D263" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E263" t="str">
+      <x:c r="E263" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F263" s="5" t="n">
@@ -13545,7 +13721,7 @@
       <x:c r="C264" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D264" t="str">
+      <x:c r="D264" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E264" t="str">
@@ -13594,10 +13770,10 @@
       <x:c r="C265" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D265" t="str">
+      <x:c r="D265" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E265" t="str">
+      <x:c r="E265" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F265" s="5" t="n">
@@ -13643,10 +13819,10 @@
       <x:c r="C266" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D266" t="str">
+      <x:c r="D266" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E266" t="str">
+      <x:c r="E266" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F266" s="5" t="n">
@@ -13692,10 +13868,10 @@
       <x:c r="C267" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D267" t="str">
+      <x:c r="D267" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E267" t="str">
+      <x:c r="E267" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F267" s="5" t="n">
@@ -13741,10 +13917,10 @@
       <x:c r="C268" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D268" t="str">
+      <x:c r="D268" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E268" t="str">
+      <x:c r="E268" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F268" s="5" t="n">
@@ -13790,7 +13966,7 @@
       <x:c r="C269" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D269" t="str">
+      <x:c r="D269" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E269" t="str">
@@ -13839,7 +14015,7 @@
       <x:c r="C270" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D270" t="str">
+      <x:c r="D270" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E270" t="str">
@@ -13888,10 +14064,10 @@
       <x:c r="C271" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D271" t="str">
+      <x:c r="D271" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E271" t="str">
+      <x:c r="E271" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F271" s="5" t="n">
@@ -13937,10 +14113,10 @@
       <x:c r="C272" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D272" t="str">
+      <x:c r="D272" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E272" t="str">
+      <x:c r="E272" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F272" s="5" t="n">
@@ -13986,7 +14162,7 @@
       <x:c r="C273" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D273" t="str">
+      <x:c r="D273" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E273" t="str">
@@ -14035,10 +14211,10 @@
       <x:c r="C274" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D274" t="str">
+      <x:c r="D274" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E274" t="str">
+      <x:c r="E274" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F274" s="5" t="n">
@@ -14084,10 +14260,10 @@
       <x:c r="C275" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D275" t="str">
+      <x:c r="D275" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E275" t="str">
+      <x:c r="E275" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F275" s="5" t="n">
@@ -14133,10 +14309,10 @@
       <x:c r="C276" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D276" t="str">
+      <x:c r="D276" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E276" t="str">
+      <x:c r="E276" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F276" s="5" t="n">
@@ -14182,7 +14358,7 @@
       <x:c r="C277" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D277" t="str">
+      <x:c r="D277" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E277" t="str">
@@ -14231,10 +14407,10 @@
       <x:c r="C278" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D278" t="str">
+      <x:c r="D278" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="E278" t="str">
+      <x:c r="E278" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="F278" s="5" t="n">
@@ -14280,10 +14456,10 @@
       <x:c r="C279" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D279" t="str">
+      <x:c r="D279" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E279" t="str">
+      <x:c r="E279" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F279" s="5" t="n">
@@ -14329,10 +14505,10 @@
       <x:c r="C280" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D280" t="str">
+      <x:c r="D280" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E280" t="str">
+      <x:c r="E280" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F280" s="5" t="n">
@@ -14378,7 +14554,7 @@
       <x:c r="C281" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D281" t="str">
+      <x:c r="D281" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E281" t="str">
@@ -14427,10 +14603,10 @@
       <x:c r="C282" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D282" t="str">
+      <x:c r="D282" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E282" t="str">
+      <x:c r="E282" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F282" s="5" t="n">
@@ -14476,10 +14652,10 @@
       <x:c r="C283" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D283" t="str">
+      <x:c r="D283" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E283" t="str">
+      <x:c r="E283" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F283" s="5" t="n">
@@ -14525,10 +14701,10 @@
       <x:c r="C284" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D284" t="str">
+      <x:c r="D284" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E284" t="str">
+      <x:c r="E284" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F284" s="5" t="n">
@@ -14574,10 +14750,10 @@
       <x:c r="C285" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D285" t="str">
+      <x:c r="D285" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E285" t="str">
+      <x:c r="E285" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F285" s="5" t="n">
@@ -14623,7 +14799,7 @@
       <x:c r="C286" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D286" t="str">
+      <x:c r="D286" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E286" t="str">
@@ -14672,10 +14848,10 @@
       <x:c r="C287" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D287" t="str">
+      <x:c r="D287" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E287" t="str">
+      <x:c r="E287" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F287" s="5" t="n">
@@ -14721,10 +14897,10 @@
       <x:c r="C288" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D288" t="str">
+      <x:c r="D288" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E288" t="str">
+      <x:c r="E288" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F288" s="5" t="n">
@@ -14770,10 +14946,10 @@
       <x:c r="C289" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D289" t="str">
+      <x:c r="D289" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E289" t="str">
+      <x:c r="E289" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F289" s="5" t="n">
@@ -14819,10 +14995,10 @@
       <x:c r="C290" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D290" t="str">
+      <x:c r="D290" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E290" t="str">
+      <x:c r="E290" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F290" s="5" t="n">
@@ -14868,10 +15044,10 @@
       <x:c r="C291" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D291" t="str">
+      <x:c r="D291" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E291" t="str">
+      <x:c r="E291" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F291" s="5" t="n">
@@ -14917,7 +15093,7 @@
       <x:c r="C292" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D292" t="str">
+      <x:c r="D292" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E292" t="str">
@@ -14966,7 +15142,7 @@
       <x:c r="C293" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D293" t="str">
+      <x:c r="D293" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E293" t="str">
@@ -15015,10 +15191,10 @@
       <x:c r="C294" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D294" t="str">
+      <x:c r="D294" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E294" t="str">
+      <x:c r="E294" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F294" s="5" t="n">
@@ -15064,10 +15240,10 @@
       <x:c r="C295" t="str">
         <x:v>25-7-2026</x:v>
       </x:c>
-      <x:c r="D295" t="str">
+      <x:c r="D295" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E295" t="str">
+      <x:c r="E295" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F295" s="5" t="n">
@@ -15113,10 +15289,10 @@
       <x:c r="C296" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D296" t="str">
+      <x:c r="D296" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E296" t="str">
+      <x:c r="E296" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F296" s="5" t="n">
@@ -15162,10 +15338,10 @@
       <x:c r="C297" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D297" t="str">
+      <x:c r="D297" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E297" t="str">
+      <x:c r="E297" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F297" s="5" t="n">
@@ -15211,7 +15387,7 @@
       <x:c r="C298" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D298" t="str">
+      <x:c r="D298" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E298" t="str">
@@ -15260,10 +15436,10 @@
       <x:c r="C299" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D299" t="str">
+      <x:c r="D299" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E299" t="str">
+      <x:c r="E299" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F299" s="5" t="n">
@@ -15309,7 +15485,7 @@
       <x:c r="C300" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D300" t="str">
+      <x:c r="D300" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E300" t="str">
@@ -15358,10 +15534,10 @@
       <x:c r="C301" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D301" t="str">
+      <x:c r="D301" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E301" t="str">
+      <x:c r="E301" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F301" s="5" t="n">
@@ -15407,10 +15583,10 @@
       <x:c r="C302" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D302" t="str">
+      <x:c r="D302" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E302" t="str">
+      <x:c r="E302" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F302" s="5" t="n">
@@ -15456,10 +15632,10 @@
       <x:c r="C303" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D303" t="str">
+      <x:c r="D303" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E303" t="str">
+      <x:c r="E303" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F303" s="5" t="n">
@@ -15505,10 +15681,10 @@
       <x:c r="C304" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D304" t="str">
+      <x:c r="D304" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E304" t="str">
+      <x:c r="E304" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F304" s="5" t="n">
@@ -15554,10 +15730,10 @@
       <x:c r="C305" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D305" t="str">
+      <x:c r="D305" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E305" t="str">
+      <x:c r="E305" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F305" s="5" t="n">
@@ -15603,10 +15779,10 @@
       <x:c r="C306" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D306" t="str">
+      <x:c r="D306" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E306" t="str">
+      <x:c r="E306" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F306" s="5" t="n">
@@ -15652,10 +15828,10 @@
       <x:c r="C307" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D307" t="str">
+      <x:c r="D307" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E307" t="str">
+      <x:c r="E307" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F307" s="5" t="n">
@@ -15701,10 +15877,10 @@
       <x:c r="C308" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D308" t="str">
+      <x:c r="D308" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E308" t="str">
+      <x:c r="E308" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F308" s="5" t="n">
@@ -15750,10 +15926,10 @@
       <x:c r="C309" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D309" t="str">
+      <x:c r="D309" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E309" t="str">
+      <x:c r="E309" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F309" s="5" t="n">
@@ -15799,10 +15975,10 @@
       <x:c r="C310" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D310" t="str">
+      <x:c r="D310" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="E310" t="str">
+      <x:c r="E310" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F310" s="5" t="n">
@@ -15850,7 +16026,7 @@
       <x:c r="C311" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D311" t="str">
+      <x:c r="D311" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E311" t="str">
@@ -15899,10 +16075,10 @@
       <x:c r="C312" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D312" t="str">
+      <x:c r="D312" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E312" t="str">
+      <x:c r="E312" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F312" s="5" t="n">
@@ -15948,7 +16124,7 @@
       <x:c r="C313" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D313" t="str">
+      <x:c r="D313" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E313" t="str">
@@ -15997,10 +16173,10 @@
       <x:c r="C314" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D314" t="str">
+      <x:c r="D314" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E314" t="str">
+      <x:c r="E314" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F314" s="5" t="n">
@@ -16046,10 +16222,10 @@
       <x:c r="C315" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D315" t="str">
+      <x:c r="D315" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E315" t="str">
+      <x:c r="E315" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F315" s="5" t="n">
@@ -16095,10 +16271,10 @@
       <x:c r="C316" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D316" t="str">
+      <x:c r="D316" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E316" t="str">
+      <x:c r="E316" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F316" s="5" t="n">
@@ -16144,10 +16320,10 @@
       <x:c r="C317" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D317" t="str">
+      <x:c r="D317" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E317" t="str">
+      <x:c r="E317" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F317" s="5" t="n">
@@ -16193,10 +16369,10 @@
       <x:c r="C318" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D318" t="str">
+      <x:c r="D318" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E318" t="str">
+      <x:c r="E318" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F318" s="5" t="n">
@@ -16242,10 +16418,10 @@
       <x:c r="C319" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D319" t="str">
+      <x:c r="D319" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E319" t="str">
+      <x:c r="E319" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F319" s="5" t="n">
@@ -16291,10 +16467,10 @@
       <x:c r="C320" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D320" t="str">
+      <x:c r="D320" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E320" t="str">
+      <x:c r="E320" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F320" s="5" t="n">
@@ -16340,10 +16516,10 @@
       <x:c r="C321" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D321" t="str">
+      <x:c r="D321" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E321" t="str">
+      <x:c r="E321" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F321" s="5" t="n">
@@ -16389,10 +16565,10 @@
       <x:c r="C322" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D322" t="str">
+      <x:c r="D322" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E322" t="str">
+      <x:c r="E322" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F322" s="5" t="n">
@@ -16438,10 +16614,10 @@
       <x:c r="C323" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D323" t="str">
+      <x:c r="D323" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E323" t="str">
+      <x:c r="E323" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F323" s="5" t="n">
@@ -16487,7 +16663,7 @@
       <x:c r="C324" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D324" t="str">
+      <x:c r="D324" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E324" t="str">
@@ -16536,10 +16712,10 @@
       <x:c r="C325" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D325" t="str">
+      <x:c r="D325" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E325" t="str">
+      <x:c r="E325" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F325" s="5" t="n">
@@ -16585,7 +16761,7 @@
       <x:c r="C326" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D326" t="str">
+      <x:c r="D326" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E326" t="str">
@@ -16634,10 +16810,10 @@
       <x:c r="C327" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D327" t="str">
+      <x:c r="D327" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E327" t="str">
+      <x:c r="E327" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F327" s="5" t="n">
@@ -16683,10 +16859,10 @@
       <x:c r="C328" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D328" t="str">
+      <x:c r="D328" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E328" t="str">
+      <x:c r="E328" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F328" s="5" t="n">
@@ -16732,10 +16908,10 @@
       <x:c r="C329" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D329" t="str">
+      <x:c r="D329" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="E329" t="str">
+      <x:c r="E329" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F329" s="5" t="n">
@@ -16781,10 +16957,10 @@
       <x:c r="C330" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D330" t="str">
+      <x:c r="D330" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E330" t="str">
+      <x:c r="E330" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F330" s="5" t="n">
@@ -16830,10 +17006,10 @@
       <x:c r="C331" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D331" t="str">
+      <x:c r="D331" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E331" t="str">
+      <x:c r="E331" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F331" s="5" t="n">
@@ -16879,10 +17055,10 @@
       <x:c r="C332" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D332" t="str">
+      <x:c r="D332" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E332" t="str">
+      <x:c r="E332" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F332" s="5" t="n">
@@ -16928,7 +17104,7 @@
       <x:c r="C333" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D333" t="str">
+      <x:c r="D333" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="E333" t="str">
@@ -17026,10 +17202,10 @@
       <x:c r="C335" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D335" t="str">
+      <x:c r="D335" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E335" t="str">
+      <x:c r="E335" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="F335" s="5" t="n">
@@ -17075,10 +17251,10 @@
       <x:c r="C336" t="str">
         <x:v>26-7-2026</x:v>
       </x:c>
-      <x:c r="D336" t="str">
+      <x:c r="D336" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="E336" t="str">
+      <x:c r="E336" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="F336" s="5" t="n">
@@ -17117,7 +17293,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cf61fe96c5b46c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0aa6f861fc74115"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17151,10 +17327,10 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="B2" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="C2" t="n">
@@ -17168,10 +17344,10 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
+      <x:c r="A3" s="20" t="str">
         <x:v>Delivery</x:v>
       </x:c>
-      <x:c r="B3" t="str">
+      <x:c r="B3" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="C3" t="n">
@@ -17185,10 +17361,10 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="A4" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="B4" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="C4" t="n">
@@ -17202,10 +17378,10 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="B5" t="str">
+      <x:c r="B5" s="35" t="str">
         <x:v>Card,Cash</x:v>
       </x:c>
       <x:c r="C5" t="n">
@@ -17219,10 +17395,10 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="C6" t="n">
@@ -17236,10 +17412,10 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="C7" t="n">
@@ -17253,7 +17429,7 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="A8" s="17" t="str">
         <x:v>Dine In</x:v>
       </x:c>
       <x:c r="B8" t="str">
@@ -17270,10 +17446,10 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="A9" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B9" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="C9" t="n">
@@ -17287,10 +17463,10 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="32" t="str">
         <x:v>Card</x:v>
       </x:c>
       <x:c r="C10" t="n">
@@ -17304,10 +17480,10 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="A11" s="14" t="str">
         <x:v>Pickup</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="29" t="str">
         <x:v>Cash</x:v>
       </x:c>
       <x:c r="C11" t="n">
@@ -17338,10 +17514,10 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="A13" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="26" t="str">
         <x:v>Keeta</x:v>
       </x:c>
       <x:c r="C13" t="n">
@@ -17355,7 +17531,7 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
+      <x:c r="A14" s="23" t="str">
         <x:v>Talabat</x:v>
       </x:c>
       <x:c r="B14" t="str">
@@ -17509,4 +17685,279 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="36" t="str">
+        <x:v>Order Type &amp; Payment Colour Standard</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="4" t="str">
+        <x:v>Channel / tender</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="str">
+        <x:v>Colour use</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="str">
+        <x:v>Control note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Dine In</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14" t="str">
+        <x:v>Pickup</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="20" t="str">
+        <x:v>Delivery</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="23" t="str">
+        <x:v>Talabat</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="39" t="str">
+        <x:v>Noon Food</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="39" t="str">
+        <x:v>Noonfood</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="42" t="str">
+        <x:v>Deliveroo</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="45" t="str">
+        <x:v>Careem</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="48" t="str">
+        <x:v>Smiles</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="26" t="str">
+        <x:v>Keeta</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>Order type</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D14" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="32" t="str">
+        <x:v>Card</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>Cash</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="35" t="str">
+        <x:v>Card,Cash</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="35" t="str">
+        <x:v>Split</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="51" t="str">
+        <x:v>Wallet</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="54" t="str">
+        <x:v>Due</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="57" t="str">
+        <x:v>Unclassified</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>Payment type</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>Same colour in dashboard, Excel and PDF</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>Red exception styling always overrides a channel colour.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>